<commit_message>
更新 default.xlsx 並移除 run.bat 暫停指令
</commit_message>
<xml_diff>
--- a/default.xlsx
+++ b/default.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\program\py\get_stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{176AC79D-9DCB-4628-8C18-494287236C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A11AFFE-EC46-471D-A630-C65684156CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="64">
   <si>
     <r>
       <rPr>
@@ -38,7 +38,7 @@
       </rPr>
       <t>日期</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -91,7 +91,7 @@
       </rPr>
       <t>漲跌</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -219,7 +219,7 @@
       </rPr>
       <t>昨收</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -257,7 +257,7 @@
       </rPr>
       <t>月</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -295,11 +295,11 @@
       </rPr>
       <t>月</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>ROE%</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -323,7 +323,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -347,7 +347,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -371,7 +371,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -395,7 +395,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -409,7 +409,7 @@
       </rPr>
       <t>每股淨值</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -444,7 +444,7 @@
       </rPr>
       <t>年</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -468,7 +468,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -492,7 +492,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -516,22 +516,22 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>利息保障
 倍數</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>應收帳款
 收現天數</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>存貨週轉
 天數</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -545,7 +545,7 @@
       </rPr>
       <t>現金股利</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -559,7 +559,7 @@
       </rPr>
       <t>股票股利</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -594,7 +594,7 @@
       </rPr>
       <t>年</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -608,7 +608,7 @@
       </rPr>
       <t>除息日</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -622,7 +622,7 @@
       </rPr>
       <t>股息發放日</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -636,7 +636,7 @@
       </rPr>
       <t>除權日</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -650,11 +650,11 @@
       </rPr>
       <t>盈餘再投資比</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>現金流</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -678,7 +678,7 @@
       </rPr>
       <t>%</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -693,12 +693,12 @@
       <t>配息
 類型</t>
     </r>
-    <phoneticPr fontId="14" type="noConversion"/>
+    <phoneticPr fontId="15" type="noConversion"/>
   </si>
   <si>
     <t>配息
 月份</t>
-    <phoneticPr fontId="14" type="noConversion"/>
+    <phoneticPr fontId="15" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -712,53 +712,126 @@
       </rPr>
       <t>代碼</t>
     </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>商品</t>
+    </r>
+  </si>
+  <si>
+    <t>0050</t>
+  </si>
+  <si>
+    <t>元大台灣50</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>半年</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>0052</t>
+  </si>
+  <si>
+    <t>富邦科技</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>年配</t>
+  </si>
+  <si>
+    <t>0056</t>
+  </si>
+  <si>
+    <t>元大高股息</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>年</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="細明體"/>
         <family val="2"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Microsoft JhengHei"/>
-        <family val="2"/>
-      </rPr>
-      <t>範例</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Tahoma"/>
-        <family val="2"/>
-      </rPr>
-      <t>)</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>商品</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+        <charset val="136"/>
+      </rPr>
+      <t>年</t>
+    </r>
+  </si>
+  <si>
+    <t>2912</t>
+  </si>
+  <si>
+    <t>統一超</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>43.87 元</t>
+  </si>
+  <si>
+    <t>3711</t>
+  </si>
+  <si>
+    <t>日月光投控</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>71.68 元</t>
+  </si>
+  <si>
+    <t>8926</t>
+  </si>
+  <si>
+    <t>台汽電</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>21.55 元</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <numFmts count="2">
+    <numFmt numFmtId="176" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="177" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
+  </numFmts>
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="新細明體"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -868,16 +941,44 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Microsoft JhengHei"/>
+      <sz val="12"/>
+      <color rgb="FF0070C0"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="12"/>
+      <color rgb="FFD60093"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="8" tint="-0.249977111117893"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
       <family val="1"/>
       <charset val="136"/>
     </font>
@@ -920,58 +1021,116 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="13" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="13" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
     <cellStyle name="一般 2" xfId="3" xr:uid="{4A0B0D9F-C1BE-476D-9649-CFB35A638A0B}"/>
+    <cellStyle name="一般 2 5" xfId="4" xr:uid="{5C832168-817F-41B2-B2CC-82C4FB9352B7}"/>
     <cellStyle name="一般 3 4" xfId="2" xr:uid="{9B84093C-831B-4D29-9B68-7EDA64845C73}"/>
     <cellStyle name="一般 59" xfId="1" xr:uid="{C1E52A47-D245-46B4-AA8F-FC0F61612BD4}"/>
   </cellStyles>
@@ -1282,44 +1441,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AP17"/>
+  <sheetFormatPr defaultColWidth="14.25" defaultRowHeight="16.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="26" max="28" width="18.25" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="14.375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="11" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17.75" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="11" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="21" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18.25" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.125" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.375" style="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.625" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="14.375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="16" width="14.375" style="13" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.625" style="13" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29" style="13" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.875" style="14" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.625" style="14" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="21" style="14" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.625" style="14" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.625" style="13" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="19.625" style="15" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="24.25" style="13" bestFit="1" customWidth="1"/>
+    <col min="29" max="31" width="20.25" style="13" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="20.625" style="13" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.75" style="13" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="18.125" style="13" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="23.75" style="13" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="17.5" style="13" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="27.125" style="13" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19.5" style="13" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="24.25" style="13" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.5" style="27" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="43" max="16384" width="14.25" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="1" customFormat="1" ht="79.2">
+    <row r="1" spans="1:42" s="1" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -1440,19 +1601,848 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:42">
-      <c r="B2">
-        <v>2330</v>
+    <row r="2" spans="1:42" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="11">
+        <v>45847</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="13">
+        <v>48</v>
+      </c>
+      <c r="E2" s="13">
+        <v>48.01</v>
+      </c>
+      <c r="F2" s="13">
+        <v>48.35</v>
+      </c>
+      <c r="G2" s="13">
+        <v>0</v>
+      </c>
+      <c r="H2" s="13">
+        <v>0</v>
+      </c>
+      <c r="I2" s="13">
+        <v>1059</v>
+      </c>
+      <c r="J2" s="13">
+        <v>112</v>
+      </c>
+      <c r="K2" s="13">
+        <v>16</v>
+      </c>
+      <c r="L2" s="13">
+        <v>0</v>
+      </c>
+      <c r="M2" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O2" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="P2" s="13">
+        <v>48.35</v>
+      </c>
+      <c r="Q2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="S2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="T2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="W2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AF2" s="13">
+        <v>2.7</v>
+      </c>
+      <c r="AG2" s="13">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="16">
+        <v>1.3599999999999999E-2</v>
+      </c>
+      <c r="AI2" s="17">
+        <v>45674</v>
+      </c>
+      <c r="AJ2" s="17">
+        <v>45877</v>
+      </c>
+      <c r="AK2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AM2" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN2" s="16">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="AO2" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="AP2" s="18" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:42">
-      <c r="B3">
+    <row r="3" spans="1:42" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
+        <v>45847</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="13">
+        <v>187.2</v>
+      </c>
+      <c r="E3" s="13">
+        <v>187.7</v>
+      </c>
+      <c r="F3" s="13">
+        <v>187.55</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0</v>
+      </c>
+      <c r="H3" s="13">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13">
+        <v>6</v>
+      </c>
+      <c r="J3" s="13">
+        <v>2</v>
+      </c>
+      <c r="K3" s="13">
+        <v>1</v>
+      </c>
+      <c r="L3" s="13">
+        <v>0</v>
+      </c>
+      <c r="M3" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O3" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="P3" s="13">
+        <v>187.55</v>
+      </c>
+      <c r="Q3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="S3" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="T3" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="W3" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="X3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AF3" s="13">
+        <v>3.23</v>
+      </c>
+      <c r="AG3" s="13">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="16">
+        <v>2.1100000000000001E-2</v>
+      </c>
+      <c r="AI3" s="17">
+        <v>45770</v>
+      </c>
+      <c r="AJ3" s="17">
+        <v>45796</v>
+      </c>
+      <c r="AK3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AM3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN3" s="16">
+        <v>1.5E-3</v>
+      </c>
+      <c r="AO3" s="20" t="s">
         <v>50</v>
       </c>
+      <c r="AP3" s="20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:42" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>45847</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="13">
+        <v>34.65</v>
+      </c>
+      <c r="E4" s="13">
+        <v>34.659999999999997</v>
+      </c>
+      <c r="F4" s="13">
+        <v>34.65</v>
+      </c>
+      <c r="G4" s="13">
+        <v>0</v>
+      </c>
+      <c r="H4" s="13">
+        <v>0</v>
+      </c>
+      <c r="I4" s="13">
+        <v>633</v>
+      </c>
+      <c r="J4" s="13">
+        <v>76</v>
+      </c>
+      <c r="K4" s="13">
+        <v>1</v>
+      </c>
+      <c r="L4" s="13">
+        <v>0</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="P4" s="13">
+        <v>34.65</v>
+      </c>
+      <c r="Q4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="R4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="S4" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="T4" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="U4" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="V4" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="W4" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="X4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AF4" s="13">
+        <v>1.07</v>
+      </c>
+      <c r="AG4" s="13">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="16">
+        <v>3.3500000000000002E-2</v>
+      </c>
+      <c r="AI4" s="17">
+        <v>45770</v>
+      </c>
+      <c r="AJ4" s="17">
+        <v>45877</v>
+      </c>
+      <c r="AK4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AM4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN4" s="16">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="AO4" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP4" s="18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>45847</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="13">
+        <v>263</v>
+      </c>
+      <c r="E5" s="13">
+        <v>263.5</v>
+      </c>
+      <c r="F5" s="13">
+        <v>263.5</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="13">
+        <v>184</v>
+      </c>
+      <c r="J5" s="13">
+        <v>4</v>
+      </c>
+      <c r="K5" s="13">
+        <v>1</v>
+      </c>
+      <c r="L5" s="13">
+        <v>0</v>
+      </c>
+      <c r="M5" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="P5" s="13">
+        <v>263.5</v>
+      </c>
+      <c r="Q5" s="13">
+        <v>23.85</v>
+      </c>
+      <c r="R5" s="13">
+        <v>6.01</v>
+      </c>
+      <c r="S5" s="22">
+        <v>6.3E-2</v>
+      </c>
+      <c r="T5" s="22">
+        <v>1.23E-2</v>
+      </c>
+      <c r="U5" s="22">
+        <v>0.33950000000000002</v>
+      </c>
+      <c r="V5" s="22">
+        <v>4.2799999999999998E-2</v>
+      </c>
+      <c r="W5" s="22">
+        <v>4.02E-2</v>
+      </c>
+      <c r="X5" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y5" s="15">
+        <v>10.210000000000001</v>
+      </c>
+      <c r="Z5" s="16">
+        <v>0.85450000000000004</v>
+      </c>
+      <c r="AA5" s="16">
+        <v>0.64590000000000003</v>
+      </c>
+      <c r="AB5" s="16">
+        <v>0.80220000000000002</v>
+      </c>
+      <c r="AC5" s="13">
+        <v>10.08</v>
+      </c>
+      <c r="AD5" s="13">
+        <v>7.42</v>
+      </c>
+      <c r="AE5" s="13">
+        <v>37.630000000000003</v>
+      </c>
+      <c r="AF5" s="13">
+        <v>9</v>
+      </c>
+      <c r="AG5" s="13">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="AI5" s="17">
+        <v>45505</v>
+      </c>
+      <c r="AJ5" s="17">
+        <v>45903</v>
+      </c>
+      <c r="AK5" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL5" s="16">
+        <v>0.58899999999999997</v>
+      </c>
+      <c r="AM5" s="23">
+        <v>-2543322</v>
+      </c>
+      <c r="AN5" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AO5" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP5" s="25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A6" s="11">
+        <v>45847</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="13">
+        <v>142.5</v>
+      </c>
+      <c r="E6" s="13">
+        <v>143</v>
+      </c>
+      <c r="F6" s="13">
+        <v>143</v>
+      </c>
+      <c r="G6" s="13">
+        <v>-1</v>
+      </c>
+      <c r="H6" s="13">
+        <v>-0.69</v>
+      </c>
+      <c r="I6" s="13">
+        <v>1005</v>
+      </c>
+      <c r="J6" s="13">
+        <v>270</v>
+      </c>
+      <c r="K6" s="13">
+        <v>83</v>
+      </c>
+      <c r="L6" s="13">
+        <v>8179</v>
+      </c>
+      <c r="M6" s="13">
+        <v>144</v>
+      </c>
+      <c r="N6" s="13">
+        <v>141.5</v>
+      </c>
+      <c r="O6" s="13">
+        <v>142.5</v>
+      </c>
+      <c r="P6" s="13">
+        <v>143</v>
+      </c>
+      <c r="Q6" s="13">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="R6" s="13">
+        <v>1.99</v>
+      </c>
+      <c r="S6" s="22">
+        <v>2.29E-2</v>
+      </c>
+      <c r="T6" s="22">
+        <v>1.03E-2</v>
+      </c>
+      <c r="U6" s="22">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="V6" s="22">
+        <v>6.5299999999999997E-2</v>
+      </c>
+      <c r="W6" s="22">
+        <v>5.2600000000000001E-2</v>
+      </c>
+      <c r="X6" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y6" s="15">
+        <v>7.51</v>
+      </c>
+      <c r="Z6" s="16">
+        <v>1.0407</v>
+      </c>
+      <c r="AA6" s="16">
+        <v>0.81720000000000004</v>
+      </c>
+      <c r="AB6" s="16">
+        <v>0.56730000000000003</v>
+      </c>
+      <c r="AC6" s="13">
+        <v>6.67</v>
+      </c>
+      <c r="AD6" s="13">
+        <v>67.78</v>
+      </c>
+      <c r="AE6" s="13">
+        <v>44.19</v>
+      </c>
+      <c r="AF6" s="13">
+        <v>5.3</v>
+      </c>
+      <c r="AG6" s="13">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="16">
+        <v>3.6400000000000002E-2</v>
+      </c>
+      <c r="AI6" s="17">
+        <v>45840</v>
+      </c>
+      <c r="AJ6" s="17">
+        <v>45868</v>
+      </c>
+      <c r="AK6" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL6" s="16">
+        <v>0.5615</v>
+      </c>
+      <c r="AM6" s="23">
+        <v>-17588099</v>
+      </c>
+      <c r="AN6" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AO6" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP6" s="25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>45847</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="13">
+        <v>42.25</v>
+      </c>
+      <c r="E7" s="13">
+        <v>42.5</v>
+      </c>
+      <c r="F7" s="13">
+        <v>42.65</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0</v>
+      </c>
+      <c r="I7" s="13">
+        <v>30</v>
+      </c>
+      <c r="J7" s="13">
+        <v>10</v>
+      </c>
+      <c r="K7" s="13">
+        <v>2</v>
+      </c>
+      <c r="L7" s="13">
+        <v>0</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="P7" s="13">
+        <v>42.65</v>
+      </c>
+      <c r="Q7" s="13">
+        <v>22.33</v>
+      </c>
+      <c r="R7" s="13">
+        <v>1.98</v>
+      </c>
+      <c r="S7" s="22">
+        <v>2.2700000000000001E-2</v>
+      </c>
+      <c r="T7" s="22">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="U7" s="22">
+        <v>0.1043</v>
+      </c>
+      <c r="V7" s="22">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="W7" s="22">
+        <v>0.1802</v>
+      </c>
+      <c r="X7" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y7" s="15">
+        <v>1.85</v>
+      </c>
+      <c r="Z7" s="16">
+        <v>0.92689999999999995</v>
+      </c>
+      <c r="AA7" s="16">
+        <v>0.92569999999999997</v>
+      </c>
+      <c r="AB7" s="16">
+        <v>0.42509999999999998</v>
+      </c>
+      <c r="AC7" s="13">
+        <v>18.829999999999998</v>
+      </c>
+      <c r="AD7" s="13">
+        <v>53.21</v>
+      </c>
+      <c r="AE7" s="13">
+        <v>0.47</v>
+      </c>
+      <c r="AF7" s="13">
+        <v>2.1</v>
+      </c>
+      <c r="AG7" s="13">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="16">
+        <v>4.7E-2</v>
+      </c>
+      <c r="AI7" s="17">
+        <v>45839</v>
+      </c>
+      <c r="AJ7" s="17">
+        <v>45863</v>
+      </c>
+      <c r="AK7" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL7" s="16">
+        <v>0.49540000000000001</v>
+      </c>
+      <c r="AM7" s="23">
+        <v>1454935</v>
+      </c>
+      <c r="AN7" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="AO7" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="AP7" s="25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+    </row>
+    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B9" s="12"/>
+    </row>
+    <row r="10" spans="1:42" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+      <c r="L10" s="29"/>
+      <c r="M10" s="29"/>
+      <c r="N10" s="29"/>
+      <c r="O10" s="29"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="29"/>
+      <c r="R10" s="29"/>
+      <c r="S10" s="30"/>
+      <c r="T10" s="30"/>
+      <c r="U10" s="30"/>
+      <c r="V10" s="30"/>
+      <c r="W10" s="30"/>
+      <c r="X10" s="31"/>
+      <c r="Y10" s="32"/>
+      <c r="Z10" s="31"/>
+      <c r="AA10" s="29"/>
+      <c r="AB10" s="31"/>
+      <c r="AC10" s="33"/>
+      <c r="AD10" s="34"/>
+      <c r="AE10" s="34"/>
+      <c r="AF10" s="31"/>
+      <c r="AG10" s="31"/>
+      <c r="AH10" s="29"/>
+      <c r="AI10" s="31"/>
+      <c r="AJ10" s="31"/>
+      <c r="AK10" s="31"/>
+      <c r="AL10" s="31"/>
+      <c r="AM10" s="35"/>
+      <c r="AN10" s="29"/>
+      <c r="AO10" s="9"/>
+      <c r="AP10" s="10"/>
+    </row>
+    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B11" s="12"/>
+    </row>
+    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B12" s="12"/>
+    </row>
+    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B13" s="19"/>
+    </row>
+    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B14" s="12"/>
+    </row>
+    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B15" s="19"/>
+    </row>
+    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="B16" s="19"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="21"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="F1:H1">
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="F1:H1048576">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -1460,7 +2450,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL1:AM1">
+  <conditionalFormatting sqref="AL1:AM1048576">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>